<commit_message>
add logo and some changes
</commit_message>
<xml_diff>
--- a/IT_Ticket_Performance_Data.xlsx
+++ b/IT_Ticket_Performance_Data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I202"/>
+  <dimension ref="A1:M215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,26 @@
           <t>Resolution_Time_Hours</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Last_Updated</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -481,12 +501,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -496,7 +516,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -505,6 +525,18 @@
       <c r="I2" t="n">
         <v>4.49</v>
       </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:22</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>TKT0001_20260407124508_test.txt,TKT0001_20260407124508_report.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -519,17 +551,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-01-30 14:17</t>
+          <t>2026-04-07 12:38</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -539,7 +571,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -548,6 +580,14 @@
       <c r="I3" t="n">
         <v>14.29</v>
       </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:38</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -582,7 +622,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -591,6 +631,14 @@
       <c r="I4" t="n">
         <v>22.93</v>
       </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:22</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -625,7 +673,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -634,6 +682,10 @@
       <c r="I5" t="n">
         <v>40.85</v>
       </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -668,7 +720,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -677,6 +729,10 @@
       <c r="I6" t="n">
         <v>43.34</v>
       </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -711,7 +767,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -720,6 +776,10 @@
       <c r="I7" t="n">
         <v>20.67</v>
       </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -754,7 +814,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -763,6 +823,10 @@
       <c r="I8" t="n">
         <v>2.88</v>
       </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -777,7 +841,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025-02-10 05:34</t>
+          <t>2026-04-02 17:55</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -787,7 +851,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -797,7 +861,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -806,6 +870,14 @@
       <c r="I9" t="n">
         <v>5.58</v>
       </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:55</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -840,7 +912,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -849,6 +921,10 @@
       <c r="I10" t="n">
         <v>31.81</v>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -883,7 +959,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -892,6 +968,10 @@
       <c r="I11" t="n">
         <v>36.16</v>
       </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -926,7 +1006,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -935,6 +1015,10 @@
       <c r="I12" t="n">
         <v>8.529999999999999</v>
       </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -969,7 +1053,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -978,6 +1062,10 @@
       <c r="I13" t="n">
         <v>46.51</v>
       </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1012,7 +1100,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -1021,6 +1109,10 @@
       <c r="I14" t="n">
         <v>19.4</v>
       </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1035,7 +1127,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2025-01-02 04:03</t>
+          <t>2026-04-02 17:05</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1045,7 +1137,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1055,7 +1147,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -1064,6 +1156,14 @@
       <c r="I15" t="n">
         <v>4.06</v>
       </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:05</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1098,7 +1198,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -1107,6 +1207,10 @@
       <c r="I16" t="n">
         <v>47.3</v>
       </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1141,7 +1245,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -1150,6 +1254,10 @@
       <c r="I17" t="n">
         <v>8.67</v>
       </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1184,7 +1292,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -1193,6 +1301,10 @@
       <c r="I18" t="n">
         <v>7.42</v>
       </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1227,7 +1339,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -1236,6 +1348,10 @@
       <c r="I19" t="n">
         <v>36.73</v>
       </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1250,7 +1366,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2025-02-22 05:39</t>
+          <t>2026-04-02 17:55</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1260,7 +1376,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1270,7 +1386,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -1279,6 +1395,14 @@
       <c r="I20" t="n">
         <v>5.66</v>
       </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:55</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1313,7 +1437,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1322,6 +1446,10 @@
       <c r="I21" t="n">
         <v>24.89</v>
       </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1356,7 +1484,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1365,6 +1493,10 @@
       <c r="I22" t="n">
         <v>27.74</v>
       </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1399,7 +1531,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1408,6 +1540,10 @@
       <c r="I23" t="n">
         <v>44.45</v>
       </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1442,7 +1578,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -1451,6 +1587,10 @@
       <c r="I24" t="n">
         <v>43.45</v>
       </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1485,7 +1625,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -1494,6 +1634,10 @@
       <c r="I25" t="n">
         <v>29.43</v>
       </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1528,7 +1672,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -1537,6 +1681,10 @@
       <c r="I26" t="n">
         <v>5.01</v>
       </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1571,7 +1719,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -1580,6 +1728,10 @@
       <c r="I27" t="n">
         <v>7.96</v>
       </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1614,7 +1766,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -1623,6 +1775,10 @@
       <c r="I28" t="n">
         <v>20.64</v>
       </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1657,7 +1813,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -1666,6 +1822,10 @@
       <c r="I29" t="n">
         <v>33.17</v>
       </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1700,7 +1860,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -1709,6 +1869,10 @@
       <c r="I30" t="n">
         <v>2.89</v>
       </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1743,7 +1907,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -1752,6 +1916,10 @@
       <c r="I31" t="n">
         <v>44.12</v>
       </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1786,7 +1954,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -1795,6 +1963,10 @@
       <c r="I32" t="n">
         <v>29.19</v>
       </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1829,7 +2001,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -1838,6 +2010,10 @@
       <c r="I33" t="n">
         <v>28.12</v>
       </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1872,7 +2048,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -1881,6 +2057,10 @@
       <c r="I34" t="n">
         <v>12.2</v>
       </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1915,7 +2095,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H35" t="n">
@@ -1924,6 +2104,10 @@
       <c r="I35" t="n">
         <v>47.89</v>
       </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1958,7 +2142,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -1967,6 +2151,10 @@
       <c r="I36" t="n">
         <v>31.73</v>
       </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2001,7 +2189,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -2010,6 +2198,10 @@
       <c r="I37" t="n">
         <v>25.94</v>
       </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2044,7 +2236,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -2053,6 +2245,10 @@
       <c r="I38" t="n">
         <v>30.98</v>
       </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2087,7 +2283,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -2096,6 +2292,10 @@
       <c r="I39" t="n">
         <v>16.68</v>
       </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2130,7 +2330,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -2139,6 +2339,10 @@
       <c r="I40" t="n">
         <v>22.32</v>
       </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2173,7 +2377,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -2182,6 +2386,10 @@
       <c r="I41" t="n">
         <v>14.72</v>
       </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2216,7 +2424,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -2225,6 +2433,10 @@
       <c r="I42" t="n">
         <v>8.119999999999999</v>
       </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2259,7 +2471,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -2268,6 +2480,10 @@
       <c r="I43" t="n">
         <v>9.83</v>
       </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2302,7 +2518,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -2311,6 +2527,10 @@
       <c r="I44" t="n">
         <v>31.37</v>
       </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2345,7 +2565,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -2354,6 +2574,10 @@
       <c r="I45" t="n">
         <v>4.52</v>
       </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2388,7 +2612,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -2397,6 +2621,10 @@
       <c r="I46" t="n">
         <v>4.71</v>
       </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2411,7 +2639,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2025-01-10 21:12</t>
+          <t>2026-04-02 17:06</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2421,7 +2649,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2431,7 +2659,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -2440,6 +2668,14 @@
       <c r="I47" t="n">
         <v>21.21</v>
       </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:06</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2474,7 +2710,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -2483,6 +2719,10 @@
       <c r="I48" t="n">
         <v>6.62</v>
       </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2517,7 +2757,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -2526,6 +2766,10 @@
       <c r="I49" t="n">
         <v>15.54</v>
       </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2560,7 +2804,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H50" t="n">
@@ -2569,6 +2813,10 @@
       <c r="I50" t="n">
         <v>39.23</v>
       </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2603,7 +2851,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H51" t="n">
@@ -2612,6 +2860,10 @@
       <c r="I51" t="n">
         <v>28.1</v>
       </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2646,7 +2898,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H52" t="n">
@@ -2655,6 +2907,10 @@
       <c r="I52" t="n">
         <v>30.63</v>
       </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2689,7 +2945,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H53" t="n">
@@ -2698,6 +2954,10 @@
       <c r="I53" t="n">
         <v>14.81</v>
       </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2732,7 +2992,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H54" t="n">
@@ -2741,6 +3001,10 @@
       <c r="I54" t="n">
         <v>23.52</v>
       </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2775,7 +3039,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H55" t="n">
@@ -2784,6 +3048,10 @@
       <c r="I55" t="n">
         <v>13.92</v>
       </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2818,7 +3086,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H56" t="n">
@@ -2827,6 +3095,10 @@
       <c r="I56" t="n">
         <v>3.66</v>
       </c>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2861,7 +3133,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -2870,6 +3142,10 @@
       <c r="I57" t="n">
         <v>12.63</v>
       </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2904,7 +3180,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H58" t="n">
@@ -2913,6 +3189,10 @@
       <c r="I58" t="n">
         <v>28.3</v>
       </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2947,7 +3227,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -2956,6 +3236,10 @@
       <c r="I59" t="n">
         <v>16.36</v>
       </c>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2990,7 +3274,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H60" t="n">
@@ -2999,6 +3283,10 @@
       <c r="I60" t="n">
         <v>35.43</v>
       </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3033,7 +3321,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -3042,6 +3330,10 @@
       <c r="I61" t="n">
         <v>35.38</v>
       </c>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3076,7 +3368,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H62" t="n">
@@ -3085,6 +3377,10 @@
       <c r="I62" t="n">
         <v>13.51</v>
       </c>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3119,7 +3415,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -3128,6 +3424,10 @@
       <c r="I63" t="n">
         <v>44.47</v>
       </c>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3162,7 +3462,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H64" t="n">
@@ -3171,6 +3471,10 @@
       <c r="I64" t="n">
         <v>26.55</v>
       </c>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3205,7 +3509,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H65" t="n">
@@ -3214,6 +3518,10 @@
       <c r="I65" t="n">
         <v>33.12</v>
       </c>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3248,7 +3556,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H66" t="n">
@@ -3257,6 +3565,10 @@
       <c r="I66" t="n">
         <v>15.2</v>
       </c>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3291,7 +3603,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H67" t="n">
@@ -3300,6 +3612,10 @@
       <c r="I67" t="n">
         <v>40.09</v>
       </c>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3334,7 +3650,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H68" t="n">
@@ -3343,6 +3659,10 @@
       <c r="I68" t="n">
         <v>34.15</v>
       </c>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3377,7 +3697,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H69" t="n">
@@ -3386,6 +3706,10 @@
       <c r="I69" t="n">
         <v>31.59</v>
       </c>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3420,7 +3744,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H70" t="n">
@@ -3429,6 +3753,10 @@
       <c r="I70" t="n">
         <v>46.05</v>
       </c>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3463,7 +3791,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H71" t="n">
@@ -3472,6 +3800,10 @@
       <c r="I71" t="n">
         <v>6.7</v>
       </c>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3506,7 +3838,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H72" t="n">
@@ -3515,6 +3847,10 @@
       <c r="I72" t="n">
         <v>7.63</v>
       </c>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3549,7 +3885,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H73" t="n">
@@ -3558,6 +3894,10 @@
       <c r="I73" t="n">
         <v>15.16</v>
       </c>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3592,7 +3932,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H74" t="n">
@@ -3601,6 +3941,10 @@
       <c r="I74" t="n">
         <v>35.33</v>
       </c>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3635,7 +3979,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H75" t="n">
@@ -3644,6 +3988,10 @@
       <c r="I75" t="n">
         <v>25.48</v>
       </c>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3678,7 +4026,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H76" t="n">
@@ -3687,6 +4035,10 @@
       <c r="I76" t="n">
         <v>12.16</v>
       </c>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3721,7 +4073,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H77" t="n">
@@ -3730,6 +4082,10 @@
       <c r="I77" t="n">
         <v>3.83</v>
       </c>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3764,7 +4120,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H78" t="n">
@@ -3773,6 +4129,10 @@
       <c r="I78" t="n">
         <v>47.91</v>
       </c>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3807,7 +4167,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H79" t="n">
@@ -3816,6 +4176,10 @@
       <c r="I79" t="n">
         <v>40.23</v>
       </c>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3850,7 +4214,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H80" t="n">
@@ -3859,6 +4223,10 @@
       <c r="I80" t="n">
         <v>5.52</v>
       </c>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3893,7 +4261,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H81" t="n">
@@ -3902,6 +4270,10 @@
       <c r="I81" t="n">
         <v>5.62</v>
       </c>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3936,7 +4308,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H82" t="n">
@@ -3945,6 +4317,10 @@
       <c r="I82" t="n">
         <v>41.99</v>
       </c>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3979,7 +4355,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -3988,6 +4364,10 @@
       <c r="I83" t="n">
         <v>34.49</v>
       </c>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4022,7 +4402,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H84" t="n">
@@ -4031,6 +4411,10 @@
       <c r="I84" t="n">
         <v>35.35</v>
       </c>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4065,7 +4449,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H85" t="n">
@@ -4074,6 +4458,10 @@
       <c r="I85" t="n">
         <v>42.42</v>
       </c>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="inlineStr"/>
+      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4108,7 +4496,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H86" t="n">
@@ -4117,6 +4505,10 @@
       <c r="I86" t="n">
         <v>36</v>
       </c>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="inlineStr"/>
+      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4151,7 +4543,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H87" t="n">
@@ -4160,6 +4552,10 @@
       <c r="I87" t="n">
         <v>24.05</v>
       </c>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4194,7 +4590,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H88" t="n">
@@ -4203,6 +4599,10 @@
       <c r="I88" t="n">
         <v>36.63</v>
       </c>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4237,7 +4637,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H89" t="n">
@@ -4246,6 +4646,10 @@
       <c r="I89" t="n">
         <v>28.89</v>
       </c>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="inlineStr"/>
+      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4280,7 +4684,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H90" t="n">
@@ -4289,6 +4693,10 @@
       <c r="I90" t="n">
         <v>46.44</v>
       </c>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4323,7 +4731,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H91" t="n">
@@ -4332,6 +4740,10 @@
       <c r="I91" t="n">
         <v>45.52</v>
       </c>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4366,7 +4778,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H92" t="n">
@@ -4375,6 +4787,10 @@
       <c r="I92" t="n">
         <v>28.33</v>
       </c>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4409,7 +4825,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H93" t="n">
@@ -4418,6 +4834,10 @@
       <c r="I93" t="n">
         <v>7.54</v>
       </c>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4452,7 +4872,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H94" t="n">
@@ -4461,6 +4881,10 @@
       <c r="I94" t="n">
         <v>41.03</v>
       </c>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4495,7 +4919,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H95" t="n">
@@ -4504,6 +4928,10 @@
       <c r="I95" t="n">
         <v>15.24</v>
       </c>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4538,7 +4966,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H96" t="n">
@@ -4547,6 +4975,10 @@
       <c r="I96" t="n">
         <v>40.16</v>
       </c>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4561,7 +4993,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2025-01-07 21:34</t>
+          <t>2026-04-02 17:54</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4571,7 +5003,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4581,7 +5013,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H97" t="n">
@@ -4590,6 +5022,14 @@
       <c r="I97" t="n">
         <v>45.58</v>
       </c>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:54</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4624,7 +5064,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H98" t="n">
@@ -4633,6 +5073,10 @@
       <c r="I98" t="n">
         <v>26.33</v>
       </c>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4667,7 +5111,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H99" t="n">
@@ -4676,6 +5120,10 @@
       <c r="I99" t="n">
         <v>38.5</v>
       </c>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr"/>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4710,7 +5158,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H100" t="n">
@@ -4719,6 +5167,10 @@
       <c r="I100" t="n">
         <v>30.47</v>
       </c>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4753,7 +5205,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H101" t="n">
@@ -4762,6 +5214,10 @@
       <c r="I101" t="n">
         <v>25.93</v>
       </c>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4796,7 +5252,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H102" t="n">
@@ -4805,6 +5261,10 @@
       <c r="I102" t="n">
         <v>36.14</v>
       </c>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4839,7 +5299,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H103" t="n">
@@ -4848,6 +5308,10 @@
       <c r="I103" t="n">
         <v>18.79</v>
       </c>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4882,7 +5346,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H104" t="n">
@@ -4891,6 +5355,10 @@
       <c r="I104" t="n">
         <v>4.56</v>
       </c>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4925,7 +5393,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H105" t="n">
@@ -4934,6 +5402,10 @@
       <c r="I105" t="n">
         <v>36.3</v>
       </c>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4968,7 +5440,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H106" t="n">
@@ -4977,6 +5449,10 @@
       <c r="I106" t="n">
         <v>15.33</v>
       </c>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5011,7 +5487,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H107" t="n">
@@ -5020,6 +5496,10 @@
       <c r="I107" t="n">
         <v>7.03</v>
       </c>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5054,7 +5534,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H108" t="n">
@@ -5063,6 +5543,10 @@
       <c r="I108" t="n">
         <v>29.43</v>
       </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5097,7 +5581,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H109" t="n">
@@ -5106,6 +5590,10 @@
       <c r="I109" t="n">
         <v>3.19</v>
       </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5140,7 +5628,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H110" t="n">
@@ -5149,6 +5637,10 @@
       <c r="I110" t="n">
         <v>9.76</v>
       </c>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5183,7 +5675,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H111" t="n">
@@ -5192,6 +5684,10 @@
       <c r="I111" t="n">
         <v>34.06</v>
       </c>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5226,7 +5722,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H112" t="n">
@@ -5235,6 +5731,10 @@
       <c r="I112" t="n">
         <v>9.07</v>
       </c>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5269,7 +5769,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H113" t="n">
@@ -5278,6 +5778,10 @@
       <c r="I113" t="n">
         <v>20.67</v>
       </c>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5312,7 +5816,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H114" t="n">
@@ -5321,6 +5825,10 @@
       <c r="I114" t="n">
         <v>2.04</v>
       </c>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5355,7 +5863,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H115" t="n">
@@ -5364,6 +5872,10 @@
       <c r="I115" t="n">
         <v>43.6</v>
       </c>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5398,7 +5910,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H116" t="n">
@@ -5407,6 +5919,10 @@
       <c r="I116" t="n">
         <v>39.46</v>
       </c>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5441,7 +5957,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H117" t="n">
@@ -5450,6 +5966,10 @@
       <c r="I117" t="n">
         <v>42.67</v>
       </c>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5484,7 +6004,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H118" t="n">
@@ -5493,6 +6013,10 @@
       <c r="I118" t="n">
         <v>8.16</v>
       </c>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5527,7 +6051,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H119" t="n">
@@ -5536,6 +6060,10 @@
       <c r="I119" t="n">
         <v>37.85</v>
       </c>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5570,7 +6098,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H120" t="n">
@@ -5579,6 +6107,10 @@
       <c r="I120" t="n">
         <v>40.99</v>
       </c>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5613,7 +6145,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H121" t="n">
@@ -5622,6 +6154,10 @@
       <c r="I121" t="n">
         <v>16.14</v>
       </c>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5656,7 +6192,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H122" t="n">
@@ -5665,6 +6201,10 @@
       <c r="I122" t="n">
         <v>5.16</v>
       </c>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5699,7 +6239,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H123" t="n">
@@ -5708,6 +6248,10 @@
       <c r="I123" t="n">
         <v>19.8</v>
       </c>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5742,7 +6286,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H124" t="n">
@@ -5751,6 +6295,10 @@
       <c r="I124" t="n">
         <v>25.46</v>
       </c>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5785,7 +6333,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H125" t="n">
@@ -5794,6 +6342,10 @@
       <c r="I125" t="n">
         <v>29.11</v>
       </c>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5828,7 +6380,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H126" t="n">
@@ -5837,6 +6389,10 @@
       <c r="I126" t="n">
         <v>6.73</v>
       </c>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5871,7 +6427,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H127" t="n">
@@ -5880,6 +6436,10 @@
       <c r="I127" t="n">
         <v>17.45</v>
       </c>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5914,7 +6474,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H128" t="n">
@@ -5923,6 +6483,10 @@
       <c r="I128" t="n">
         <v>9.51</v>
       </c>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5957,7 +6521,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H129" t="n">
@@ -5966,6 +6530,10 @@
       <c r="I129" t="n">
         <v>36.43</v>
       </c>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6000,7 +6568,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H130" t="n">
@@ -6009,6 +6577,10 @@
       <c r="I130" t="n">
         <v>46.41</v>
       </c>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6043,7 +6615,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H131" t="n">
@@ -6052,6 +6624,10 @@
       <c r="I131" t="n">
         <v>46.61</v>
       </c>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6086,7 +6662,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H132" t="n">
@@ -6095,6 +6671,10 @@
       <c r="I132" t="n">
         <v>14.53</v>
       </c>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6129,7 +6709,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H133" t="n">
@@ -6138,6 +6718,10 @@
       <c r="I133" t="n">
         <v>25.74</v>
       </c>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6172,7 +6756,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H134" t="n">
@@ -6181,6 +6765,10 @@
       <c r="I134" t="n">
         <v>25.11</v>
       </c>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6215,7 +6803,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H135" t="n">
@@ -6224,6 +6812,10 @@
       <c r="I135" t="n">
         <v>33.21</v>
       </c>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr"/>
+      <c r="L135" t="inlineStr"/>
+      <c r="M135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6258,7 +6850,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H136" t="n">
@@ -6267,6 +6859,10 @@
       <c r="I136" t="n">
         <v>42.22</v>
       </c>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr"/>
+      <c r="L136" t="inlineStr"/>
+      <c r="M136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6281,7 +6877,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2025-01-19 20:56</t>
+          <t>2026-04-02 17:06</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -6291,7 +6887,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -6301,7 +6897,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H137" t="n">
@@ -6310,6 +6906,14 @@
       <c r="I137" t="n">
         <v>44.94</v>
       </c>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:06</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6344,7 +6948,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H138" t="n">
@@ -6353,6 +6957,10 @@
       <c r="I138" t="n">
         <v>24.06</v>
       </c>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr"/>
+      <c r="L138" t="inlineStr"/>
+      <c r="M138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6387,7 +6995,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H139" t="n">
@@ -6396,6 +7004,10 @@
       <c r="I139" t="n">
         <v>21.65</v>
       </c>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr"/>
+      <c r="L139" t="inlineStr"/>
+      <c r="M139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6430,7 +7042,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H140" t="n">
@@ -6439,6 +7051,10 @@
       <c r="I140" t="n">
         <v>29.29</v>
       </c>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr"/>
+      <c r="L140" t="inlineStr"/>
+      <c r="M140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6473,7 +7089,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H141" t="n">
@@ -6482,6 +7098,10 @@
       <c r="I141" t="n">
         <v>3.58</v>
       </c>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6516,7 +7136,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H142" t="n">
@@ -6525,6 +7145,10 @@
       <c r="I142" t="n">
         <v>2.94</v>
       </c>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr"/>
+      <c r="L142" t="inlineStr"/>
+      <c r="M142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6559,7 +7183,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H143" t="n">
@@ -6568,6 +7192,10 @@
       <c r="I143" t="n">
         <v>22.07</v>
       </c>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr"/>
+      <c r="L143" t="inlineStr"/>
+      <c r="M143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6602,7 +7230,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H144" t="n">
@@ -6611,6 +7239,10 @@
       <c r="I144" t="n">
         <v>47.42</v>
       </c>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr"/>
+      <c r="M144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6645,7 +7277,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H145" t="n">
@@ -6654,6 +7286,10 @@
       <c r="I145" t="n">
         <v>5.56</v>
       </c>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6688,7 +7324,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H146" t="n">
@@ -6697,6 +7333,10 @@
       <c r="I146" t="n">
         <v>32.58</v>
       </c>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr"/>
+      <c r="M146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6731,7 +7371,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H147" t="n">
@@ -6740,6 +7380,10 @@
       <c r="I147" t="n">
         <v>38.24</v>
       </c>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6774,7 +7418,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H148" t="n">
@@ -6783,6 +7427,10 @@
       <c r="I148" t="n">
         <v>21.35</v>
       </c>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr"/>
+      <c r="M148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6817,7 +7465,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H149" t="n">
@@ -6826,6 +7474,10 @@
       <c r="I149" t="n">
         <v>15.04</v>
       </c>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr"/>
+      <c r="M149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6860,7 +7512,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H150" t="n">
@@ -6869,6 +7521,10 @@
       <c r="I150" t="n">
         <v>15.54</v>
       </c>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr"/>
+      <c r="M150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6903,7 +7559,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H151" t="n">
@@ -6912,6 +7568,10 @@
       <c r="I151" t="n">
         <v>16.82</v>
       </c>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr"/>
+      <c r="M151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6946,7 +7606,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H152" t="n">
@@ -6955,6 +7615,10 @@
       <c r="I152" t="n">
         <v>7.66</v>
       </c>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6989,7 +7653,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H153" t="n">
@@ -6998,6 +7662,10 @@
       <c r="I153" t="n">
         <v>4.08</v>
       </c>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7032,7 +7700,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H154" t="n">
@@ -7041,6 +7709,10 @@
       <c r="I154" t="n">
         <v>2.11</v>
       </c>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr"/>
+      <c r="M154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7075,7 +7747,7 @@
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H155" t="n">
@@ -7084,6 +7756,10 @@
       <c r="I155" t="n">
         <v>45.58</v>
       </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr"/>
+      <c r="M155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -7098,7 +7774,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2025-01-16 22:42</t>
+          <t>2026-04-02 17:06</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -7108,7 +7784,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -7118,7 +7794,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H156" t="n">
@@ -7127,6 +7803,14 @@
       <c r="I156" t="n">
         <v>46.7</v>
       </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:06</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7161,7 +7845,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H157" t="n">
@@ -7170,6 +7854,10 @@
       <c r="I157" t="n">
         <v>26.54</v>
       </c>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr"/>
+      <c r="M157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7204,7 +7892,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H158" t="n">
@@ -7213,6 +7901,10 @@
       <c r="I158" t="n">
         <v>8.9</v>
       </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr"/>
+      <c r="M158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7247,7 +7939,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H159" t="n">
@@ -7256,6 +7948,10 @@
       <c r="I159" t="n">
         <v>27.22</v>
       </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr"/>
+      <c r="M159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7290,7 +7986,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H160" t="n">
@@ -7299,6 +7995,10 @@
       <c r="I160" t="n">
         <v>25.57</v>
       </c>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr"/>
+      <c r="M160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -7333,7 +8033,7 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H161" t="n">
@@ -7342,6 +8042,10 @@
       <c r="I161" t="n">
         <v>38.38</v>
       </c>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr"/>
+      <c r="M161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -7376,7 +8080,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H162" t="n">
@@ -7385,6 +8089,10 @@
       <c r="I162" t="n">
         <v>27.17</v>
       </c>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr"/>
+      <c r="M162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -7419,7 +8127,7 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H163" t="n">
@@ -7428,6 +8136,10 @@
       <c r="I163" t="n">
         <v>39.58</v>
       </c>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr"/>
+      <c r="M163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -7462,7 +8174,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H164" t="n">
@@ -7471,6 +8183,10 @@
       <c r="I164" t="n">
         <v>44.67</v>
       </c>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr"/>
+      <c r="L164" t="inlineStr"/>
+      <c r="M164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7505,7 +8221,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H165" t="n">
@@ -7514,6 +8230,10 @@
       <c r="I165" t="n">
         <v>6.93</v>
       </c>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
+      <c r="L165" t="inlineStr"/>
+      <c r="M165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7548,7 +8268,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H166" t="n">
@@ -7557,6 +8277,10 @@
       <c r="I166" t="n">
         <v>29.53</v>
       </c>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr"/>
+      <c r="L166" t="inlineStr"/>
+      <c r="M166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7591,7 +8315,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H167" t="n">
@@ -7600,6 +8324,10 @@
       <c r="I167" t="n">
         <v>21.48</v>
       </c>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr"/>
+      <c r="L167" t="inlineStr"/>
+      <c r="M167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -7634,7 +8362,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H168" t="n">
@@ -7643,6 +8371,10 @@
       <c r="I168" t="n">
         <v>37.46</v>
       </c>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr"/>
+      <c r="M168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -7677,7 +8409,7 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H169" t="n">
@@ -7686,6 +8418,10 @@
       <c r="I169" t="n">
         <v>20.81</v>
       </c>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr"/>
+      <c r="M169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7720,7 +8456,7 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H170" t="n">
@@ -7729,6 +8465,10 @@
       <c r="I170" t="n">
         <v>43.95</v>
       </c>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr"/>
+      <c r="M170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7763,7 +8503,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H171" t="n">
@@ -7772,6 +8512,10 @@
       <c r="I171" t="n">
         <v>12.07</v>
       </c>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr"/>
+      <c r="M171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7806,7 +8550,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H172" t="n">
@@ -7815,6 +8559,10 @@
       <c r="I172" t="n">
         <v>18.74</v>
       </c>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="inlineStr"/>
+      <c r="M172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -7849,7 +8597,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H173" t="n">
@@ -7858,6 +8606,10 @@
       <c r="I173" t="n">
         <v>28.92</v>
       </c>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7892,7 +8644,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H174" t="n">
@@ -7901,6 +8653,10 @@
       <c r="I174" t="n">
         <v>6.34</v>
       </c>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7935,7 +8691,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H175" t="n">
@@ -7944,6 +8700,10 @@
       <c r="I175" t="n">
         <v>38.71</v>
       </c>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -7978,7 +8738,7 @@
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H176" t="n">
@@ -7987,6 +8747,10 @@
       <c r="I176" t="n">
         <v>31.96</v>
       </c>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8021,7 +8785,7 @@
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H177" t="n">
@@ -8030,6 +8794,10 @@
       <c r="I177" t="n">
         <v>39.26</v>
       </c>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8064,7 +8832,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H178" t="n">
@@ -8073,6 +8841,10 @@
       <c r="I178" t="n">
         <v>32.44</v>
       </c>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8107,7 +8879,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H179" t="n">
@@ -8116,6 +8888,10 @@
       <c r="I179" t="n">
         <v>21.72</v>
       </c>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8150,7 +8926,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H180" t="n">
@@ -8159,6 +8935,10 @@
       <c r="I180" t="n">
         <v>28.17</v>
       </c>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -8193,7 +8973,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H181" t="n">
@@ -8202,6 +8982,10 @@
       <c r="I181" t="n">
         <v>8.83</v>
       </c>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr"/>
+      <c r="M181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -8236,7 +9020,7 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H182" t="n">
@@ -8245,6 +9029,10 @@
       <c r="I182" t="n">
         <v>29.41</v>
       </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -8279,7 +9067,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H183" t="n">
@@ -8288,6 +9076,10 @@
       <c r="I183" t="n">
         <v>30.8</v>
       </c>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr"/>
+      <c r="M183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -8322,7 +9114,7 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H184" t="n">
@@ -8331,6 +9123,10 @@
       <c r="I184" t="n">
         <v>34.9</v>
       </c>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -8365,7 +9161,7 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H185" t="n">
@@ -8374,6 +9170,10 @@
       <c r="I185" t="n">
         <v>36.23</v>
       </c>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -8408,7 +9208,7 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H186" t="n">
@@ -8417,6 +9217,10 @@
       <c r="I186" t="n">
         <v>15.95</v>
       </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -8451,7 +9255,7 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H187" t="n">
@@ -8460,6 +9264,10 @@
       <c r="I187" t="n">
         <v>37.26</v>
       </c>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr"/>
+      <c r="M187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -8494,7 +9302,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Agent_D</t>
+          <t>agent.dana@it.com</t>
         </is>
       </c>
       <c r="H188" t="n">
@@ -8503,6 +9311,10 @@
       <c r="I188" t="n">
         <v>33</v>
       </c>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
+      <c r="L188" t="inlineStr"/>
+      <c r="M188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -8537,7 +9349,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H189" t="n">
@@ -8546,6 +9358,10 @@
       <c r="I189" t="n">
         <v>22.73</v>
       </c>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr"/>
+      <c r="M189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -8580,7 +9396,7 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H190" t="n">
@@ -8589,6 +9405,10 @@
       <c r="I190" t="n">
         <v>44.5</v>
       </c>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr"/>
+      <c r="L190" t="inlineStr"/>
+      <c r="M190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -8623,7 +9443,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H191" t="n">
@@ -8632,6 +9452,10 @@
       <c r="I191" t="n">
         <v>27.13</v>
       </c>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr"/>
+      <c r="L191" t="inlineStr"/>
+      <c r="M191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8666,7 +9490,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H192" t="n">
@@ -8675,6 +9499,10 @@
       <c r="I192" t="n">
         <v>11.5</v>
       </c>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -8709,7 +9537,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Agent_B</t>
+          <t>agent.blake@it.com</t>
         </is>
       </c>
       <c r="H193" t="n">
@@ -8718,6 +9546,10 @@
       <c r="I193" t="n">
         <v>23.7</v>
       </c>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr"/>
+      <c r="L193" t="inlineStr"/>
+      <c r="M193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -8752,7 +9584,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H194" t="n">
@@ -8761,6 +9593,10 @@
       <c r="I194" t="n">
         <v>5.15</v>
       </c>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr"/>
+      <c r="L194" t="inlineStr"/>
+      <c r="M194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8795,7 +9631,7 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H195" t="n">
@@ -8804,6 +9640,10 @@
       <c r="I195" t="n">
         <v>3.95</v>
       </c>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr"/>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -8838,7 +9678,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H196" t="n">
@@ -8847,6 +9687,10 @@
       <c r="I196" t="n">
         <v>40.26</v>
       </c>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr"/>
+      <c r="L196" t="inlineStr"/>
+      <c r="M196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -8881,7 +9725,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H197" t="n">
@@ -8890,6 +9734,10 @@
       <c r="I197" t="n">
         <v>47.17</v>
       </c>
+      <c r="J197" t="inlineStr"/>
+      <c r="K197" t="inlineStr"/>
+      <c r="L197" t="inlineStr"/>
+      <c r="M197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8924,7 +9772,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H198" t="n">
@@ -8933,6 +9781,10 @@
       <c r="I198" t="n">
         <v>25.17</v>
       </c>
+      <c r="J198" t="inlineStr"/>
+      <c r="K198" t="inlineStr"/>
+      <c r="L198" t="inlineStr"/>
+      <c r="M198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -8967,7 +9819,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Agent_A</t>
+          <t>agent.alex@it.com</t>
         </is>
       </c>
       <c r="H199" t="n">
@@ -8976,6 +9828,10 @@
       <c r="I199" t="n">
         <v>29.7</v>
       </c>
+      <c r="J199" t="inlineStr"/>
+      <c r="K199" t="inlineStr"/>
+      <c r="L199" t="inlineStr"/>
+      <c r="M199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -9010,7 +9866,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H200" t="n">
@@ -9019,6 +9875,10 @@
       <c r="I200" t="n">
         <v>35.85</v>
       </c>
+      <c r="J200" t="inlineStr"/>
+      <c r="K200" t="inlineStr"/>
+      <c r="L200" t="inlineStr"/>
+      <c r="M200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -9053,7 +9913,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H201" t="n">
@@ -9062,6 +9922,10 @@
       <c r="I201" t="n">
         <v>5.55</v>
       </c>
+      <c r="J201" t="inlineStr"/>
+      <c r="K201" t="inlineStr"/>
+      <c r="L201" t="inlineStr"/>
+      <c r="M201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9096,7 +9960,7 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>Agent_C</t>
+          <t>agent.chris@it.com</t>
         </is>
       </c>
       <c r="H202" t="n">
@@ -9105,6 +9969,707 @@
       <c r="I202" t="n">
         <v>5.55</v>
       </c>
+      <c r="J202" t="inlineStr"/>
+      <c r="K202" t="inlineStr"/>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>TKT-20260402-5756</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:51</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:06</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>agent.alex@it.com</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr"/>
+      <c r="I203" t="inlineStr"/>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>my printer is out of ink</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:06</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>TKT-20260402-1499</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:51</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:06</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>agent.alex@it.com</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr"/>
+      <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>my printer is out of ink</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:06</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>TKT-20260402-6653</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:51</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>agent.alex@it.com</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr"/>
+      <c r="I205" t="inlineStr"/>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>my printer is out of ink</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>TKT-20260402-9102</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:51</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>agent.alex@it.com</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr"/>
+      <c r="I206" t="inlineStr"/>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>my printer is out of ink</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>TKT-20260402-3073</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:51</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>agent.alex@it.com</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr"/>
+      <c r="I207" t="inlineStr"/>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>my printer is out of ink</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>TKT-20260402-1239</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:51</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>agent.alex@it.com</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr"/>
+      <c r="I208" t="inlineStr"/>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>my printer is out of ink</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:07</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>TKT-20260402-2009</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-04-02 16:51</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:20</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>admin@it.com</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr"/>
+      <c r="I209" t="inlineStr"/>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>my printer is out of ink</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>2026-04-02 17:20</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>TKT-20260402-8156</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:07</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr"/>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>agent.dana@it.com</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr"/>
+      <c r="I210" t="inlineStr"/>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>malekaroza8765@gmail.com</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>facing network issue</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>2026-04-02 18:07</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>TKT-20260407-3365</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-04-07 11:34</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr"/>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>agent.dana@it.com</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr"/>
+      <c r="I211" t="inlineStr"/>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>admin@it.com</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Test ticket for debugging
+--- Auto-merged duplicates ---
+[From TKT-20260407-2344] Test ticket for debugging</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:21</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>TKT-20260407-6577</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-04-07 11:35</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr"/>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>agent.dana@it.com</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr"/>
+      <c r="I212" t="inlineStr"/>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>admin@it.com</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Test ticket for debugging</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>2026-04-07 11:35</t>
+        </is>
+      </c>
+      <c r="M212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>TKT-20260407-3487</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:20</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr"/>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr"/>
+      <c r="I213" t="inlineStr"/>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>admin@it.com</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Test ticket for debugging</t>
+        </is>
+      </c>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:20</t>
+        </is>
+      </c>
+      <c r="M213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>TKT-20260407-2344</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:21</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:21</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr"/>
+      <c r="I214" t="inlineStr"/>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>admin@it.com</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Test ticket for debugging</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:21</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>TKT-20260407-2334</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:38</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr"/>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr"/>
+      <c r="I215" t="inlineStr"/>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>admin@it.com</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Outlook not syncing emails properly</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>2026-04-07 12:38</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>